<commit_message>
Support EAN and UPC identifier modes
</commit_message>
<xml_diff>
--- a/public/templates/url-generator-eans-template.xlsx
+++ b/public/templates/url-generator-eans-template.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="17">
   <si>
     <t>product</t>
   </si>
@@ -19,6 +19,12 @@
     <t>ean</t>
   </si>
   <si>
+    <t>upc</t>
+  </si>
+  <si>
+    <t>mode</t>
+  </si>
+  <si>
     <t>sku</t>
   </si>
   <si>
@@ -28,7 +34,34 @@
     <t>0123456789012</t>
   </si>
   <si>
+    <t/>
+  </si>
+  <si>
     <t>SKU-ABC-123</t>
+  </si>
+  <si>
+    <t>DEF-456</t>
+  </si>
+  <si>
+    <t>1234567890123</t>
+  </si>
+  <si>
+    <t>123456789012</t>
+  </si>
+  <si>
+    <t>SKU-DEF-456</t>
+  </si>
+  <si>
+    <t>GHI-789</t>
+  </si>
+  <si>
+    <t>987654321098</t>
+  </si>
+  <si>
+    <t>upc only</t>
+  </si>
+  <si>
+    <t>SKU-GHI-789</t>
   </si>
 </sst>
 </file>
@@ -73,11 +106,21 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -417,36 +460,86 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="3" width="14" style="1" customWidth="1"/>
+    <col min="1" max="1" width="18" style="1" customWidth="1"/>
+    <col min="2" max="2" width="18" style="2" customWidth="1"/>
+    <col min="3" max="3" width="16" style="2" customWidth="1"/>
+    <col min="4" max="4" width="14" style="1" customWidth="1"/>
+    <col min="5" max="5" width="18" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
+      <c r="D1" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>4</v>
+      </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="1" t="s">
         <v>5</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C2"/>
+  <autoFilter ref="A1:E4"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>